<commit_message>
Describe reachability stratification in appendix
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/kiribati_tb_modelling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B062981-514D-1E46-B866-AD395ADF49E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79AB1B22-6D59-964E-A33A-B842FEC6CB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7120" yWindow="1480" windowWidth="38400" windowHeight="21100" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="145">
   <si>
     <t>parameter</t>
   </si>
@@ -1220,9 +1220,6 @@
       <c r="G14" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="I14" s="5" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="15" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">

</xml_diff>

<commit_message>
Separate sensitivity parameters in different table
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/kiribati_tb_modelling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79AB1B22-6D59-964E-A33A-B842FEC6CB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB1A1B0-8578-D340-BDE9-C7F8DBFAF71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7120" yWindow="1480" windowWidth="38400" windowHeight="21100" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
   <sheets>
     <sheet name="constant" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="147">
   <si>
     <t>parameter</t>
   </si>
@@ -472,6 +472,12 @@
   </si>
   <si>
     <t>Probability of TST positivity for 'contained' state</t>
+  </si>
+  <si>
+    <t>skip</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -940,7 +946,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57F6C8F8-7718-2F41-B98B-2D455BE12E8B}">
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
@@ -953,7 +959,7 @@
     <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -981,8 +987,11 @@
       <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="J1" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
@@ -1005,7 +1014,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>129</v>
       </c>
@@ -1025,7 +1034,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>127</v>
       </c>
@@ -1048,7 +1057,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>128</v>
       </c>
@@ -1071,7 +1080,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
@@ -1094,7 +1103,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
@@ -1117,7 +1126,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>22</v>
       </c>
@@ -1140,7 +1149,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>19</v>
       </c>
@@ -1151,7 +1160,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>54</v>
       </c>
@@ -1165,7 +1174,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>61</v>
       </c>
@@ -1182,7 +1191,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>62</v>
       </c>
@@ -1196,7 +1205,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>63</v>
       </c>
@@ -1210,7 +1219,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>67</v>
       </c>
@@ -1221,7 +1230,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>64</v>
       </c>
@@ -1238,7 +1247,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>65</v>
       </c>
@@ -1551,7 +1560,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="33" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
         <v>57</v>
       </c>
@@ -1562,7 +1571,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
         <v>58</v>
       </c>
@@ -1573,7 +1582,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="35" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
         <v>50</v>
       </c>
@@ -1584,7 +1593,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
         <v>51</v>
       </c>
@@ -1595,7 +1604,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="37" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="10" t="s">
         <v>103</v>
       </c>
@@ -1605,8 +1614,11 @@
       <c r="G37" s="10" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="J37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
         <v>104</v>
       </c>
@@ -1616,8 +1628,11 @@
       <c r="G38" s="10" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="J38" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
         <v>105</v>
       </c>
@@ -1627,8 +1642,11 @@
       <c r="G39" s="10" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="J39" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
         <v>106</v>
       </c>
@@ -1638,8 +1656,11 @@
       <c r="G40" s="10" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="J40" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>59</v>
       </c>
@@ -1659,7 +1680,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="42" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>60</v>
       </c>
@@ -1670,7 +1691,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
         <v>52</v>
       </c>
@@ -1690,7 +1711,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="44" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
         <v>53</v>
       </c>
@@ -1701,7 +1722,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
         <v>111</v>
       </c>
@@ -1712,7 +1733,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
         <v>112</v>
       </c>
@@ -1723,7 +1744,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
         <v>113</v>
       </c>
@@ -1734,7 +1755,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="48" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
         <v>114</v>
       </c>
@@ -1745,7 +1766,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="49" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="8" t="s">
         <v>49</v>
       </c>
@@ -1759,7 +1780,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>20</v>
       </c>
@@ -1769,8 +1790,11 @@
       <c r="G50" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J50" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>119</v>
       </c>
@@ -1790,7 +1814,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>121</v>
       </c>
@@ -1801,7 +1825,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>123</v>
       </c>
@@ -1821,7 +1845,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>125</v>
       </c>
@@ -1841,7 +1865,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>133</v>
       </c>
@@ -1852,7 +1876,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>135</v>
       </c>
@@ -1863,7 +1887,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>137</v>
       </c>

</xml_diff>

<commit_message>
Include lit review and references
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/kiribati_tb_modelling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB1A1B0-8578-D340-BDE9-C7F8DBFAF71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D1DEBC-701D-0743-A5F7-6BF392F8CF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="147">
   <si>
     <t>parameter</t>
   </si>
@@ -1229,6 +1229,9 @@
       <c r="G14" s="5" t="s">
         <v>77</v>
       </c>
+      <c r="J14" s="5" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="15" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">

</xml_diff>

<commit_message>
Rename parameters to include units
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/kiribati_tb_modelling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D1DEBC-701D-0743-A5F7-6BF392F8CF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCB0804-EBA1-764A-9E77-6C954C2C0FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -261,60 +261,12 @@
     <t>Rel. infectiousness of 'less infectious' TB (ref. 'more infectious' TB)</t>
   </si>
   <si>
-    <t>Rate of progression from 'incipient' to TB disease (age 0-4)</t>
-  </si>
-  <si>
-    <t>Rate of progression from 'incipient' to TB disease (age 5-14)</t>
-  </si>
-  <si>
-    <t>Rate of progression from 'incipient' to TB disease (age 15 and over)</t>
-  </si>
-  <si>
     <t>Proportion of incident TB that is 'more infectious'</t>
   </si>
   <si>
-    <t>Rate of transition from 'incipient' to 'contained' (age 0-4)</t>
-  </si>
-  <si>
-    <t>Rate of transition from 'incipient' to 'contained' (age 5-14)</t>
-  </si>
-  <si>
-    <t>Rate of transition from 'incipient' to 'contained' (age 15 and over)</t>
-  </si>
-  <si>
-    <t>Rate of transition from 'contained' to 'incipient' (all ages)</t>
-  </si>
-  <si>
-    <t>Rate of transition from 'contained' to 'cleared' (all ages)</t>
-  </si>
-  <si>
-    <t>Rate of progression from subclinical to clinical TB</t>
-  </si>
-  <si>
-    <t>Rate of transition from clinical to subclinical TB</t>
-  </si>
-  <si>
-    <t>Rate of progression from 'less infectious' to 'more infectious' TB</t>
-  </si>
-  <si>
-    <t>Rate of transition from 'more infectious' to 'less infectious' TB</t>
-  </si>
-  <si>
-    <t>Rate of TB mortality for 'more infectious' clinical disease</t>
-  </si>
-  <si>
-    <t>Rate of TB mortality for 'less infectious' clinical disease</t>
-  </si>
-  <si>
-    <t>Rate of self-recovery for subclinical TB</t>
-  </si>
-  <si>
     <t>Annual rate of TB detection in 2020</t>
   </si>
   <si>
-    <t>Average TB treatment duration</t>
-  </si>
-  <si>
     <t>Percentage of deaths among negative TB treatment outcomes</t>
   </si>
   <si>
@@ -478,6 +430,54 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Average TB treatment duration (years)</t>
+  </si>
+  <si>
+    <t>Rate of self-recovery for subclinical TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of TB mortality for 'less infectious' clinical disease (/year)</t>
+  </si>
+  <si>
+    <t>Rate of TB mortality for 'more infectious' clinical disease (/year)</t>
+  </si>
+  <si>
+    <t>Rate of transition from 'more infectious' to 'less infectious' TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of progression from 'less infectious' to 'more infectious' TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of transition from clinical to subclinical TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of progression from subclinical to clinical TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of transition from 'contained' to 'cleared' (all ages, /year)</t>
+  </si>
+  <si>
+    <t>Rate of transition from 'contained' to 'incipient' (all ages, /year)</t>
+  </si>
+  <si>
+    <t>Rate of transition from 'incipient' to 'contained' (age 15 and over, /year)</t>
+  </si>
+  <si>
+    <t>Rate of transition from 'incipient' to 'contained' (age 5-14, /year)</t>
+  </si>
+  <si>
+    <t>Rate of transition from 'incipient' to 'contained' (age 0-4, /year)</t>
+  </si>
+  <si>
+    <t>Rate of progression from 'incipient' to TB disease (age 15 and over, /year)</t>
+  </si>
+  <si>
+    <t>Rate of progression from 'incipient' to TB disease (age 5-14, /year)</t>
+  </si>
+  <si>
+    <t>Rate of progression from 'incipient' to TB disease (age 0-4, /year)</t>
   </si>
 </sst>
 </file>
@@ -988,7 +988,7 @@
         <v>24</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -1016,7 +1016,7 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="B3" s="2">
         <v>0.05</v>
@@ -1031,12 +1031,12 @@
         <v>0.05</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1051,7 +1051,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>28</v>
@@ -1059,7 +1059,7 @@
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="B5" s="2">
         <v>0.2</v>
@@ -1074,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>29</v>
@@ -1182,7 +1182,7 @@
         <v>2.4</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>74</v>
+        <v>146</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>34</v>
@@ -1199,7 +1199,7 @@
         <v>2</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>25</v>
@@ -1213,7 +1213,7 @@
         <v>0.1</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>76</v>
+        <v>144</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>25</v>
@@ -1227,10 +1227,10 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -1241,7 +1241,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>78</v>
+        <v>143</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>35</v>
@@ -1258,7 +1258,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>79</v>
+        <v>142</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>25</v>
@@ -1272,7 +1272,7 @@
         <v>2</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>80</v>
+        <v>141</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>25</v>
@@ -1295,7 +1295,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>81</v>
+        <v>140</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>36</v>
@@ -1321,7 +1321,7 @@
         <v>0.1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>82</v>
+        <v>139</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>39</v>
@@ -1347,7 +1347,7 @@
         <v>5</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>83</v>
+        <v>138</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>40</v>
@@ -1364,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>84</v>
+        <v>137</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>41</v>
@@ -1390,7 +1390,7 @@
         <v>10</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>85</v>
+        <v>136</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>42</v>
@@ -1407,7 +1407,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>86</v>
+        <v>135</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>43</v>
@@ -1424,7 +1424,7 @@
         <v>0.38900000000000001</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>87</v>
+        <v>134</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>38</v>
@@ -1441,7 +1441,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>88</v>
+        <v>133</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>56</v>
@@ -1458,7 +1458,7 @@
         <v>0.4</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>37</v>
@@ -1484,7 +1484,7 @@
         <v>5</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>25</v>
@@ -1498,7 +1498,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>91</v>
+        <v>131</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>48</v>
@@ -1515,7 +1515,7 @@
         <v>40</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>44</v>
@@ -1523,29 +1523,29 @@
     </row>
     <row r="30" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="B30" s="5">
         <v>0.75</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="B31" s="5">
         <v>0.75</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="B32" s="5">
         <v>0.35</v>
@@ -1560,7 +1560,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1571,7 +1571,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1582,7 +1582,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1593,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1604,63 +1604,63 @@
         <v>1</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="10" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="B37" s="10">
         <v>0.3</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="J37" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B38" s="10">
         <v>1</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="J38" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
     </row>
     <row r="39" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="B39" s="10">
         <v>0.5</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="J39" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
     </row>
     <row r="40" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="B40" s="10">
         <v>1</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="J40" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
     </row>
     <row r="41" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1680,7 +1680,7 @@
         <v>0.52</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1691,7 +1691,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1711,7 +1711,7 @@
         <v>0.93</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1722,51 +1722,51 @@
         <v>1</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="B45" s="12">
         <v>0</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="B46" s="12">
         <v>1</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
     </row>
     <row r="47" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="B47" s="12">
         <v>0</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="B48" s="12">
         <v>1</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -1777,7 +1777,7 @@
         <v>70</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>44</v>
@@ -1791,15 +1791,15 @@
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="J50" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="B51" s="13">
         <v>2000</v>
@@ -1814,23 +1814,23 @@
         <v>2020</v>
       </c>
       <c r="G51" s="13" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="B52" s="13">
         <v>0.15</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="B53">
         <v>0.5</v>
@@ -1845,12 +1845,12 @@
         <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="B54">
         <v>0.5</v>
@@ -1865,40 +1865,40 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="B55">
         <v>0.85</v>
       </c>
       <c r="G55" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="B56">
         <v>0.5</v>
       </c>
       <c r="G56" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="B57">
         <v>1.5</v>
       </c>
       <c r="G57" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More progress on appendix
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/kiribati_tb_modelling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCB0804-EBA1-764A-9E77-6C954C2C0FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3511CEF-02A0-E249-B44D-A8105751CA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -252,9 +252,6 @@
     <t>Rel. susceptibility to infection for under 15 year-old individuals (ref. 15 and over)</t>
   </si>
   <si>
-    <t>Rel. risk of reinfection from 'cleared' compartment (ref. 'mtb-naïve')</t>
-  </si>
-  <si>
     <t>Rel. infectiousness of subclinical TB (ref. clinical TB)</t>
   </si>
   <si>
@@ -267,9 +264,6 @@
     <t>Annual rate of TB detection in 2020</t>
   </si>
   <si>
-    <t>Percentage of deaths among negative TB treatment outcomes</t>
-  </si>
-  <si>
     <t>Probability PEARL-positive for 'subclinical' and 'less infectious' category</t>
   </si>
   <si>
@@ -351,9 +345,6 @@
     <t>passive_detection_inflection</t>
   </si>
   <si>
-    <t>Time when passive detection started to scale up</t>
-  </si>
-  <si>
     <t>passive_detection_shape</t>
   </si>
   <si>
@@ -369,9 +360,6 @@
     <t>infection_pop_scale</t>
   </si>
   <si>
-    <t>Exponent for population scaling in force of infection calculation</t>
-  </si>
-  <si>
     <t>a_spread</t>
   </si>
   <si>
@@ -399,15 +387,9 @@
     <t>rel_detection_unreachable</t>
   </si>
   <si>
-    <t>Relative detection rate of unreachable population under passive case finding (ref. reachable)</t>
-  </si>
-  <si>
     <t>rel_sus_unreachable</t>
   </si>
   <si>
-    <t>Relative susceptibility to infection of unreachable population (ref. reachable)</t>
-  </si>
-  <si>
     <t>prev_se_incipient_tst</t>
   </si>
   <si>
@@ -444,15 +426,9 @@
     <t>Rate of TB mortality for 'more infectious' clinical disease (/year)</t>
   </si>
   <si>
-    <t>Rate of transition from 'more infectious' to 'less infectious' TB (/year)</t>
-  </si>
-  <si>
     <t>Rate of progression from 'less infectious' to 'more infectious' TB (/year)</t>
   </si>
   <si>
-    <t>Rate of transition from clinical to subclinical TB (/year)</t>
-  </si>
-  <si>
     <t>Rate of progression from subclinical to clinical TB (/year)</t>
   </si>
   <si>
@@ -478,6 +454,30 @@
   </si>
   <si>
     <t>Rate of progression from 'incipient' to TB disease (age 0-4, /year)</t>
+  </si>
+  <si>
+    <t>Population-size exponent in the force of infection, from density-dependent (0) to frequency-dependent (1) transmission</t>
+  </si>
+  <si>
+    <t>Rel. risk of reinfection from 'cleared' and 'recovered' compartment (ref. 'mtb-naïve')</t>
+  </si>
+  <si>
+    <t>Rate of regression from clinical to subclinical TB (/year)</t>
+  </si>
+  <si>
+    <t>Rate of regression from 'more infectious' to 'less infectious' TB (/year)</t>
+  </si>
+  <si>
+    <t>Percentage of deaths among non-successful TB treatment outcomes</t>
+  </si>
+  <si>
+    <t>Inflection year of the passive detection scale-up profile</t>
+  </si>
+  <si>
+    <t>Relative detection rate of hard-to-reach population under passive case finding (ref. screening-reachable)</t>
+  </si>
+  <si>
+    <t>Relative susceptibility to infection of hard-to-reach population (ref. screening-reachable)</t>
   </si>
 </sst>
 </file>
@@ -988,7 +988,7 @@
         <v>24</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -1016,7 +1016,7 @@
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B3" s="2">
         <v>0.05</v>
@@ -1031,12 +1031,12 @@
         <v>0.05</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1051,7 +1051,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>28</v>
@@ -1059,7 +1059,7 @@
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B5" s="2">
         <v>0.2</v>
@@ -1074,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>29</v>
@@ -1120,7 +1120,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>71</v>
+        <v>140</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>31</v>
@@ -1157,7 +1157,7 @@
         <v>0.5</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1168,7 +1168,7 @@
         <v>0.4</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>33</v>
@@ -1182,7 +1182,7 @@
         <v>2.4</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>34</v>
@@ -1199,7 +1199,7 @@
         <v>2</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>25</v>
@@ -1213,7 +1213,7 @@
         <v>0.1</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>25</v>
@@ -1227,10 +1227,10 @@
         <v>0.5</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -1241,7 +1241,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>35</v>
@@ -1258,7 +1258,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>25</v>
@@ -1272,7 +1272,7 @@
         <v>2</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>25</v>
@@ -1295,7 +1295,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>36</v>
@@ -1321,7 +1321,7 @@
         <v>0.1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>39</v>
@@ -1347,7 +1347,7 @@
         <v>5</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>40</v>
@@ -1364,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>41</v>
@@ -1390,7 +1390,7 @@
         <v>10</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>42</v>
@@ -1407,7 +1407,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>43</v>
@@ -1424,7 +1424,7 @@
         <v>0.38900000000000001</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>38</v>
@@ -1441,7 +1441,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>56</v>
@@ -1458,7 +1458,7 @@
         <v>0.4</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>37</v>
@@ -1484,7 +1484,7 @@
         <v>5</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>25</v>
@@ -1498,7 +1498,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>48</v>
@@ -1515,7 +1515,7 @@
         <v>40</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>76</v>
+        <v>143</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>44</v>
@@ -1523,29 +1523,29 @@
     </row>
     <row r="30" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B30" s="5">
         <v>0.75</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B31" s="5">
         <v>0.75</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B32" s="5">
         <v>0.35</v>
@@ -1560,7 +1560,7 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1571,7 +1571,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1582,7 +1582,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1593,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -1604,63 +1604,63 @@
         <v>1</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B37" s="10">
         <v>0.3</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J37" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B38" s="10">
         <v>1</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J38" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="39" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B39" s="10">
         <v>0.5</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J39" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="40" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B40" s="10">
         <v>1</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J40" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="41" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1680,7 +1680,7 @@
         <v>0.52</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1691,7 +1691,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1711,7 +1711,7 @@
         <v>0.93</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
@@ -1722,51 +1722,51 @@
         <v>1</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B45" s="12">
         <v>0</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B46" s="12">
         <v>1</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B47" s="12">
         <v>0</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B48" s="12">
         <v>1</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -1777,7 +1777,7 @@
         <v>70</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>44</v>
@@ -1791,15 +1791,15 @@
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J50" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B51" s="13">
         <v>2000</v>
@@ -1814,23 +1814,23 @@
         <v>2020</v>
       </c>
       <c r="G51" s="13" t="s">
-        <v>104</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B52" s="13">
         <v>0.15</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B53">
         <v>0.5</v>
@@ -1845,12 +1845,12 @@
         <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B54">
         <v>0.5</v>
@@ -1865,40 +1865,40 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>110</v>
+        <v>139</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B55">
         <v>0.85</v>
       </c>
       <c r="G55" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B56">
         <v>0.5</v>
       </c>
       <c r="G56" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B57">
         <v>1.5</v>
       </c>
       <c r="G57" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>